<commit_message>
FWD: date drop-downs in the workbook, explicit phase-1/phase-2 send buttons
</commit_message>
<xml_diff>
--- a/docs/templates/FWD_ACTUAL_sample_P1.xlsx
+++ b/docs/templates/FWD_ACTUAL_sample_P1.xlsx
@@ -5,7 +5,8 @@
   <workbookPr defaultThemeVersion="164011" filterPrivacy="1"/>
   <sheets>
     <sheet sheetId="1" name="FWD_ACTUAL" state="visible" r:id="rId4"/>
-    <sheet sheetId="2" name="README" state="visible" r:id="rId5"/>
+    <sheet sheetId="2" name="DATES" state="veryHidden" r:id="rId5"/>
+    <sheet sheetId="3" name="README" state="visible" r:id="rId6"/>
   </sheets>
   <calcPr calcId="171027"/>
 </workbook>
@@ -83,7 +84,7 @@
     <t/>
   </si>
   <si>
-    <t>YYYY-MM-DD</t>
+    <t>pick from list · dd-mmm-yyyy</t>
   </si>
   <si>
     <t>THB/kg</t>
@@ -161,7 +162,7 @@
     <t>text</t>
   </si>
   <si>
-    <t>date — YYYY-MM-DD · e.g. YYYY-MM-DD</t>
+    <t>date — pick from the drop-down (dd-mmm-yyyy) · e.g. pick from list · dd-mmm-yyyy</t>
   </si>
   <si>
     <t>number (no currency symbol) · e.g. THB/kg</t>
@@ -183,6 +184,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="dd-mmm-yyyy"/>
+  </numFmts>
   <fonts count="4" x14ac:knownFonts="1">
     <font>
       <color theme="1"/>
@@ -259,20 +263,26 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="164" fontId="1" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="164" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="0" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
@@ -632,8 +642,8 @@
     <col min="9" max="10" width="13" customWidth="1"/>
     <col min="11" max="11" width="32" customWidth="1"/>
     <col min="12" max="13" width="16" customWidth="1"/>
-    <col min="14" max="15" width="13" customWidth="1"/>
-    <col min="16" max="16" width="18" customWidth="1"/>
+    <col min="14" max="15" width="13" style="1" customWidth="1"/>
+    <col min="16" max="16" width="18" style="1" customWidth="1"/>
     <col min="17" max="17" width="19" customWidth="1"/>
     <col min="18" max="18" width="18" customWidth="1"/>
     <col min="19" max="19" width="23" customWidth="1"/>
@@ -643,207 +653,1726 @@
   </cols>
   <sheetData>
     <row r="1" ht="32" customHeight="1" spans="1:22" x14ac:dyDescent="0.25">
-      <c r="A1" s="1" t="s">
+      <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="H1" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="I1" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="J1" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="K1" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="2" t="s">
+      <c r="L1" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="M1" s="2" t="s">
+      <c r="M1" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="N1" s="2" t="s">
+      <c r="N1" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="O1" s="2" t="s">
+      <c r="O1" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="P1" s="2" t="s">
+      <c r="P1" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" s="2" t="s">
+      <c r="Q1" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="R1" s="2" t="s">
+      <c r="R1" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="S1" s="3" t="s">
+      <c r="S1" s="5" t="s">
         <v>18</v>
       </c>
-      <c r="T1" s="3" t="s">
+      <c r="T1" s="5" t="s">
         <v>19</v>
       </c>
-      <c r="U1" s="3" t="s">
+      <c r="U1" s="5" t="s">
         <v>20</v>
       </c>
-      <c r="V1" s="1" t="s">
+      <c r="V1" s="2" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="2" spans="1:22" s="4" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="4" t="s">
-        <v>22</v>
-      </c>
-      <c r="B2" s="4" t="s">
-        <v>22</v>
-      </c>
-      <c r="C2" s="4" t="s">
-        <v>22</v>
-      </c>
-      <c r="D2" s="4" t="s">
-        <v>22</v>
-      </c>
-      <c r="E2" s="4" t="s">
-        <v>22</v>
-      </c>
-      <c r="F2" s="4" t="s">
-        <v>22</v>
-      </c>
-      <c r="G2" s="4" t="s">
-        <v>22</v>
-      </c>
-      <c r="H2" s="4" t="s">
-        <v>22</v>
-      </c>
-      <c r="I2" s="4" t="s">
-        <v>22</v>
-      </c>
-      <c r="J2" s="4" t="s">
-        <v>22</v>
-      </c>
-      <c r="K2" s="4" t="s">
-        <v>22</v>
-      </c>
-      <c r="L2" s="4" t="s">
-        <v>22</v>
-      </c>
-      <c r="M2" s="4" t="s">
-        <v>22</v>
-      </c>
-      <c r="N2" s="4" t="s">
+    <row r="2" spans="1:22" s="6" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A2" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="B2" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="C2" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="D2" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="E2" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="F2" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="G2" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="H2" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="I2" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="J2" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="K2" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="L2" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="M2" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="N2" s="7" t="s">
         <v>23</v>
       </c>
-      <c r="O2" s="4" t="s">
+      <c r="O2" s="7" t="s">
         <v>23</v>
       </c>
-      <c r="P2" s="4" t="s">
+      <c r="P2" s="7" t="s">
         <v>23</v>
       </c>
-      <c r="Q2" s="4" t="s">
+      <c r="Q2" s="6" t="s">
         <v>24</v>
       </c>
-      <c r="R2" s="4" t="s">
-        <v>22</v>
-      </c>
-      <c r="S2" s="4" t="s">
+      <c r="R2" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="S2" s="6" t="s">
         <v>25</v>
       </c>
-      <c r="T2" s="4" t="s">
+      <c r="T2" s="6" t="s">
         <v>25</v>
       </c>
-      <c r="U2" s="4" t="s">
+      <c r="U2" s="6" t="s">
         <v>25</v>
       </c>
-      <c r="V2" s="4" t="s">
+      <c r="V2" s="6" t="s">
         <v>22</v>
       </c>
     </row>
     <row r="3" spans="1:22" x14ac:dyDescent="0.25">
-      <c r="A3" s="5" t="s">
+      <c r="A3" s="8" t="s">
         <v>26</v>
       </c>
-      <c r="B3" s="5" t="s">
+      <c r="B3" s="8" t="s">
         <v>27</v>
       </c>
-      <c r="C3" s="5" t="s">
+      <c r="C3" s="8" t="s">
         <v>28</v>
       </c>
-      <c r="D3" s="5" t="s">
+      <c r="D3" s="8" t="s">
         <v>29</v>
       </c>
-      <c r="E3" s="5" t="s">
+      <c r="E3" s="8" t="s">
         <v>30</v>
       </c>
-      <c r="F3" s="5" t="s">
+      <c r="F3" s="8" t="s">
         <v>31</v>
       </c>
-      <c r="G3" s="5">
+      <c r="G3" s="8">
         <v>42.67</v>
       </c>
-      <c r="H3" s="5" t="s">
+      <c r="H3" s="8" t="s">
         <v>32</v>
       </c>
-      <c r="I3" s="5" t="s">
+      <c r="I3" s="8" t="s">
         <v>33</v>
       </c>
-      <c r="J3" s="5" t="s">
+      <c r="J3" s="8" t="s">
         <v>34</v>
       </c>
-      <c r="K3" s="5" t="s">
+      <c r="K3" s="8" t="s">
         <v>35</v>
       </c>
-      <c r="L3" s="6" t="s">
-        <v>22</v>
-      </c>
-      <c r="M3" s="6" t="s">
-        <v>22</v>
-      </c>
-      <c r="N3" s="6" t="s">
-        <v>22</v>
-      </c>
-      <c r="O3" s="6" t="s">
-        <v>22</v>
-      </c>
-      <c r="P3" s="6" t="s">
-        <v>22</v>
-      </c>
-      <c r="Q3" s="6" t="s">
-        <v>22</v>
-      </c>
-      <c r="R3" s="6" t="s">
-        <v>22</v>
-      </c>
-      <c r="S3" s="7" t="s">
-        <v>22</v>
-      </c>
-      <c r="T3" s="7" t="s">
-        <v>22</v>
-      </c>
-      <c r="U3" s="7" t="s">
-        <v>22</v>
-      </c>
-      <c r="V3" s="5" t="s">
+      <c r="L3" s="9" t="s">
+        <v>22</v>
+      </c>
+      <c r="M3" s="9" t="s">
+        <v>22</v>
+      </c>
+      <c r="N3" s="10" t="s">
+        <v>22</v>
+      </c>
+      <c r="O3" s="10" t="s">
+        <v>22</v>
+      </c>
+      <c r="P3" s="10" t="s">
+        <v>22</v>
+      </c>
+      <c r="Q3" s="9" t="s">
+        <v>22</v>
+      </c>
+      <c r="R3" s="9" t="s">
+        <v>22</v>
+      </c>
+      <c r="S3" s="11" t="s">
+        <v>22</v>
+      </c>
+      <c r="T3" s="11" t="s">
+        <v>22</v>
+      </c>
+      <c r="U3" s="11" t="s">
+        <v>22</v>
+      </c>
+      <c r="V3" s="8" t="s">
         <v>36</v>
+      </c>
+    </row>
+  </sheetData>
+  <dataValidations count="1">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" promptTitle="Date" prompt="Click the arrow and pick a date (dd-mmm-yyyy)." showErrorMessage="1" errorStyle="warning" errorTitle="Pick a date" error="Please choose a date from the drop-down (dd-mmm-yyyy, e.g. 23-Sep-2026)." sqref="N3:P3">
+      <formula1>=DATES!$A$1:$A$300</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:A300"/>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <cols>
+    <col min="1" max="1" width="16" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A1" s="1">
+        <v>46272.70833333333</v>
+      </c>
+    </row>
+    <row r="2" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A2" s="1">
+        <v>46273.70833333333</v>
+      </c>
+    </row>
+    <row r="3" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A3" s="1">
+        <v>46274.70833333333</v>
+      </c>
+    </row>
+    <row r="4" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A4" s="1">
+        <v>46275.70833333333</v>
+      </c>
+    </row>
+    <row r="5" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A5" s="1">
+        <v>46276.70833333333</v>
+      </c>
+    </row>
+    <row r="6" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A6" s="1">
+        <v>46277.70833333333</v>
+      </c>
+    </row>
+    <row r="7" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A7" s="1">
+        <v>46278.70833333333</v>
+      </c>
+    </row>
+    <row r="8" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A8" s="1">
+        <v>46279.70833333333</v>
+      </c>
+    </row>
+    <row r="9" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A9" s="1">
+        <v>46280.70833333333</v>
+      </c>
+    </row>
+    <row r="10" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A10" s="1">
+        <v>46281.70833333333</v>
+      </c>
+    </row>
+    <row r="11" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A11" s="1">
+        <v>46282.70833333333</v>
+      </c>
+    </row>
+    <row r="12" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A12" s="1">
+        <v>46283.70833333333</v>
+      </c>
+    </row>
+    <row r="13" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A13" s="1">
+        <v>46284.70833333333</v>
+      </c>
+    </row>
+    <row r="14" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A14" s="1">
+        <v>46285.70833333333</v>
+      </c>
+    </row>
+    <row r="15" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A15" s="1">
+        <v>46286.70833333333</v>
+      </c>
+    </row>
+    <row r="16" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A16" s="1">
+        <v>46287.70833333333</v>
+      </c>
+    </row>
+    <row r="17" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A17" s="1">
+        <v>46288.70833333333</v>
+      </c>
+    </row>
+    <row r="18" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A18" s="1">
+        <v>46289.70833333333</v>
+      </c>
+    </row>
+    <row r="19" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A19" s="1">
+        <v>46290.70833333333</v>
+      </c>
+    </row>
+    <row r="20" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A20" s="1">
+        <v>46291.70833333333</v>
+      </c>
+    </row>
+    <row r="21" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A21" s="1">
+        <v>46292.70833333333</v>
+      </c>
+    </row>
+    <row r="22" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A22" s="1">
+        <v>46293.70833333333</v>
+      </c>
+    </row>
+    <row r="23" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A23" s="1">
+        <v>46294.70833333333</v>
+      </c>
+    </row>
+    <row r="24" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A24" s="1">
+        <v>46295.70833333333</v>
+      </c>
+    </row>
+    <row r="25" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A25" s="1">
+        <v>46296.70833333333</v>
+      </c>
+    </row>
+    <row r="26" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A26" s="1">
+        <v>46297.70833333333</v>
+      </c>
+    </row>
+    <row r="27" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A27" s="1">
+        <v>46298.70833333333</v>
+      </c>
+    </row>
+    <row r="28" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A28" s="1">
+        <v>46299.70833333333</v>
+      </c>
+    </row>
+    <row r="29" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A29" s="1">
+        <v>46300.70833333333</v>
+      </c>
+    </row>
+    <row r="30" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A30" s="1">
+        <v>46301.70833333333</v>
+      </c>
+    </row>
+    <row r="31" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A31" s="1">
+        <v>46302.70833333333</v>
+      </c>
+    </row>
+    <row r="32" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A32" s="1">
+        <v>46303.70833333333</v>
+      </c>
+    </row>
+    <row r="33" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A33" s="1">
+        <v>46304.70833333333</v>
+      </c>
+    </row>
+    <row r="34" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A34" s="1">
+        <v>46305.70833333333</v>
+      </c>
+    </row>
+    <row r="35" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A35" s="1">
+        <v>46306.70833333333</v>
+      </c>
+    </row>
+    <row r="36" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A36" s="1">
+        <v>46307.70833333333</v>
+      </c>
+    </row>
+    <row r="37" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A37" s="1">
+        <v>46308.70833333333</v>
+      </c>
+    </row>
+    <row r="38" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A38" s="1">
+        <v>46309.70833333333</v>
+      </c>
+    </row>
+    <row r="39" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A39" s="1">
+        <v>46310.70833333333</v>
+      </c>
+    </row>
+    <row r="40" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A40" s="1">
+        <v>46311.70833333333</v>
+      </c>
+    </row>
+    <row r="41" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A41" s="1">
+        <v>46312.70833333333</v>
+      </c>
+    </row>
+    <row r="42" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A42" s="1">
+        <v>46313.70833333333</v>
+      </c>
+    </row>
+    <row r="43" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A43" s="1">
+        <v>46314.70833333333</v>
+      </c>
+    </row>
+    <row r="44" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A44" s="1">
+        <v>46315.70833333333</v>
+      </c>
+    </row>
+    <row r="45" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A45" s="1">
+        <v>46316.70833333333</v>
+      </c>
+    </row>
+    <row r="46" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A46" s="1">
+        <v>46317.70833333333</v>
+      </c>
+    </row>
+    <row r="47" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A47" s="1">
+        <v>46318.70833333333</v>
+      </c>
+    </row>
+    <row r="48" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A48" s="1">
+        <v>46319.70833333333</v>
+      </c>
+    </row>
+    <row r="49" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A49" s="1">
+        <v>46320.70833333333</v>
+      </c>
+    </row>
+    <row r="50" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A50" s="1">
+        <v>46321.70833333333</v>
+      </c>
+    </row>
+    <row r="51" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A51" s="1">
+        <v>46322.70833333333</v>
+      </c>
+    </row>
+    <row r="52" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A52" s="1">
+        <v>46323.70833333333</v>
+      </c>
+    </row>
+    <row r="53" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A53" s="1">
+        <v>46324.70833333333</v>
+      </c>
+    </row>
+    <row r="54" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A54" s="1">
+        <v>46325.70833333333</v>
+      </c>
+    </row>
+    <row r="55" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A55" s="1">
+        <v>46326.70833333333</v>
+      </c>
+    </row>
+    <row r="56" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A56" s="1">
+        <v>46327.70833333333</v>
+      </c>
+    </row>
+    <row r="57" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A57" s="1">
+        <v>46328.70833333333</v>
+      </c>
+    </row>
+    <row r="58" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A58" s="1">
+        <v>46329.70833333333</v>
+      </c>
+    </row>
+    <row r="59" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A59" s="1">
+        <v>46330.70833333333</v>
+      </c>
+    </row>
+    <row r="60" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A60" s="1">
+        <v>46331.70833333333</v>
+      </c>
+    </row>
+    <row r="61" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A61" s="1">
+        <v>46332.70833333333</v>
+      </c>
+    </row>
+    <row r="62" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A62" s="1">
+        <v>46333.70833333333</v>
+      </c>
+    </row>
+    <row r="63" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A63" s="1">
+        <v>46334.70833333333</v>
+      </c>
+    </row>
+    <row r="64" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A64" s="1">
+        <v>46335.70833333333</v>
+      </c>
+    </row>
+    <row r="65" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A65" s="1">
+        <v>46336.70833333333</v>
+      </c>
+    </row>
+    <row r="66" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A66" s="1">
+        <v>46337.70833333333</v>
+      </c>
+    </row>
+    <row r="67" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A67" s="1">
+        <v>46338.70833333333</v>
+      </c>
+    </row>
+    <row r="68" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A68" s="1">
+        <v>46339.70833333333</v>
+      </c>
+    </row>
+    <row r="69" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A69" s="1">
+        <v>46340.70833333333</v>
+      </c>
+    </row>
+    <row r="70" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A70" s="1">
+        <v>46341.70833333333</v>
+      </c>
+    </row>
+    <row r="71" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A71" s="1">
+        <v>46342.70833333333</v>
+      </c>
+    </row>
+    <row r="72" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A72" s="1">
+        <v>46343.70833333333</v>
+      </c>
+    </row>
+    <row r="73" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A73" s="1">
+        <v>46344.70833333333</v>
+      </c>
+    </row>
+    <row r="74" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A74" s="1">
+        <v>46345.70833333333</v>
+      </c>
+    </row>
+    <row r="75" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A75" s="1">
+        <v>46346.70833333333</v>
+      </c>
+    </row>
+    <row r="76" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A76" s="1">
+        <v>46347.70833333333</v>
+      </c>
+    </row>
+    <row r="77" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A77" s="1">
+        <v>46348.70833333333</v>
+      </c>
+    </row>
+    <row r="78" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A78" s="1">
+        <v>46349.70833333333</v>
+      </c>
+    </row>
+    <row r="79" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A79" s="1">
+        <v>46350.70833333333</v>
+      </c>
+    </row>
+    <row r="80" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A80" s="1">
+        <v>46351.70833333333</v>
+      </c>
+    </row>
+    <row r="81" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A81" s="1">
+        <v>46352.70833333333</v>
+      </c>
+    </row>
+    <row r="82" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A82" s="1">
+        <v>46353.70833333333</v>
+      </c>
+    </row>
+    <row r="83" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A83" s="1">
+        <v>46354.70833333333</v>
+      </c>
+    </row>
+    <row r="84" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A84" s="1">
+        <v>46355.70833333333</v>
+      </c>
+    </row>
+    <row r="85" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A85" s="1">
+        <v>46356.70833333333</v>
+      </c>
+    </row>
+    <row r="86" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A86" s="1">
+        <v>46357.70833333333</v>
+      </c>
+    </row>
+    <row r="87" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A87" s="1">
+        <v>46358.70833333333</v>
+      </c>
+    </row>
+    <row r="88" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A88" s="1">
+        <v>46359.70833333333</v>
+      </c>
+    </row>
+    <row r="89" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A89" s="1">
+        <v>46360.70833333333</v>
+      </c>
+    </row>
+    <row r="90" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A90" s="1">
+        <v>46361.70833333333</v>
+      </c>
+    </row>
+    <row r="91" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A91" s="1">
+        <v>46362.70833333333</v>
+      </c>
+    </row>
+    <row r="92" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A92" s="1">
+        <v>46363.70833333333</v>
+      </c>
+    </row>
+    <row r="93" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A93" s="1">
+        <v>46364.70833333333</v>
+      </c>
+    </row>
+    <row r="94" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A94" s="1">
+        <v>46365.70833333333</v>
+      </c>
+    </row>
+    <row r="95" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A95" s="1">
+        <v>46366.70833333333</v>
+      </c>
+    </row>
+    <row r="96" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A96" s="1">
+        <v>46367.70833333333</v>
+      </c>
+    </row>
+    <row r="97" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A97" s="1">
+        <v>46368.70833333333</v>
+      </c>
+    </row>
+    <row r="98" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A98" s="1">
+        <v>46369.70833333333</v>
+      </c>
+    </row>
+    <row r="99" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A99" s="1">
+        <v>46370.70833333333</v>
+      </c>
+    </row>
+    <row r="100" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A100" s="1">
+        <v>46371.70833333333</v>
+      </c>
+    </row>
+    <row r="101" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A101" s="1">
+        <v>46372.70833333333</v>
+      </c>
+    </row>
+    <row r="102" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A102" s="1">
+        <v>46373.70833333333</v>
+      </c>
+    </row>
+    <row r="103" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A103" s="1">
+        <v>46374.70833333333</v>
+      </c>
+    </row>
+    <row r="104" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A104" s="1">
+        <v>46375.70833333333</v>
+      </c>
+    </row>
+    <row r="105" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A105" s="1">
+        <v>46376.70833333333</v>
+      </c>
+    </row>
+    <row r="106" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A106" s="1">
+        <v>46377.70833333333</v>
+      </c>
+    </row>
+    <row r="107" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A107" s="1">
+        <v>46378.70833333333</v>
+      </c>
+    </row>
+    <row r="108" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A108" s="1">
+        <v>46379.70833333333</v>
+      </c>
+    </row>
+    <row r="109" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A109" s="1">
+        <v>46380.70833333333</v>
+      </c>
+    </row>
+    <row r="110" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A110" s="1">
+        <v>46381.70833333333</v>
+      </c>
+    </row>
+    <row r="111" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A111" s="1">
+        <v>46382.70833333333</v>
+      </c>
+    </row>
+    <row r="112" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A112" s="1">
+        <v>46383.70833333333</v>
+      </c>
+    </row>
+    <row r="113" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A113" s="1">
+        <v>46384.70833333333</v>
+      </c>
+    </row>
+    <row r="114" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A114" s="1">
+        <v>46385.70833333333</v>
+      </c>
+    </row>
+    <row r="115" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A115" s="1">
+        <v>46386.70833333333</v>
+      </c>
+    </row>
+    <row r="116" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A116" s="1">
+        <v>46387.70833333333</v>
+      </c>
+    </row>
+    <row r="117" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A117" s="1">
+        <v>46388.70833333333</v>
+      </c>
+    </row>
+    <row r="118" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A118" s="1">
+        <v>46389.70833333333</v>
+      </c>
+    </row>
+    <row r="119" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A119" s="1">
+        <v>46390.70833333333</v>
+      </c>
+    </row>
+    <row r="120" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A120" s="1">
+        <v>46391.70833333333</v>
+      </c>
+    </row>
+    <row r="121" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A121" s="1">
+        <v>46392.70833333333</v>
+      </c>
+    </row>
+    <row r="122" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A122" s="1">
+        <v>46393.70833333333</v>
+      </c>
+    </row>
+    <row r="123" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A123" s="1">
+        <v>46394.70833333333</v>
+      </c>
+    </row>
+    <row r="124" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A124" s="1">
+        <v>46395.70833333333</v>
+      </c>
+    </row>
+    <row r="125" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A125" s="1">
+        <v>46396.70833333333</v>
+      </c>
+    </row>
+    <row r="126" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A126" s="1">
+        <v>46397.70833333333</v>
+      </c>
+    </row>
+    <row r="127" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A127" s="1">
+        <v>46398.70833333333</v>
+      </c>
+    </row>
+    <row r="128" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A128" s="1">
+        <v>46399.70833333333</v>
+      </c>
+    </row>
+    <row r="129" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A129" s="1">
+        <v>46400.70833333333</v>
+      </c>
+    </row>
+    <row r="130" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A130" s="1">
+        <v>46401.70833333333</v>
+      </c>
+    </row>
+    <row r="131" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A131" s="1">
+        <v>46402.70833333333</v>
+      </c>
+    </row>
+    <row r="132" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A132" s="1">
+        <v>46403.70833333333</v>
+      </c>
+    </row>
+    <row r="133" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A133" s="1">
+        <v>46404.70833333333</v>
+      </c>
+    </row>
+    <row r="134" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A134" s="1">
+        <v>46405.70833333333</v>
+      </c>
+    </row>
+    <row r="135" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A135" s="1">
+        <v>46406.70833333333</v>
+      </c>
+    </row>
+    <row r="136" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A136" s="1">
+        <v>46407.70833333333</v>
+      </c>
+    </row>
+    <row r="137" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A137" s="1">
+        <v>46408.70833333333</v>
+      </c>
+    </row>
+    <row r="138" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A138" s="1">
+        <v>46409.70833333333</v>
+      </c>
+    </row>
+    <row r="139" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A139" s="1">
+        <v>46410.70833333333</v>
+      </c>
+    </row>
+    <row r="140" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A140" s="1">
+        <v>46411.70833333333</v>
+      </c>
+    </row>
+    <row r="141" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A141" s="1">
+        <v>46412.70833333333</v>
+      </c>
+    </row>
+    <row r="142" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A142" s="1">
+        <v>46413.70833333333</v>
+      </c>
+    </row>
+    <row r="143" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A143" s="1">
+        <v>46414.70833333333</v>
+      </c>
+    </row>
+    <row r="144" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A144" s="1">
+        <v>46415.70833333333</v>
+      </c>
+    </row>
+    <row r="145" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A145" s="1">
+        <v>46416.70833333333</v>
+      </c>
+    </row>
+    <row r="146" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A146" s="1">
+        <v>46417.70833333333</v>
+      </c>
+    </row>
+    <row r="147" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A147" s="1">
+        <v>46418.70833333333</v>
+      </c>
+    </row>
+    <row r="148" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A148" s="1">
+        <v>46419.70833333333</v>
+      </c>
+    </row>
+    <row r="149" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A149" s="1">
+        <v>46420.70833333333</v>
+      </c>
+    </row>
+    <row r="150" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A150" s="1">
+        <v>46421.70833333333</v>
+      </c>
+    </row>
+    <row r="151" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A151" s="1">
+        <v>46422.70833333333</v>
+      </c>
+    </row>
+    <row r="152" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A152" s="1">
+        <v>46423.70833333333</v>
+      </c>
+    </row>
+    <row r="153" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A153" s="1">
+        <v>46424.70833333333</v>
+      </c>
+    </row>
+    <row r="154" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A154" s="1">
+        <v>46425.70833333333</v>
+      </c>
+    </row>
+    <row r="155" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A155" s="1">
+        <v>46426.70833333333</v>
+      </c>
+    </row>
+    <row r="156" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A156" s="1">
+        <v>46427.70833333333</v>
+      </c>
+    </row>
+    <row r="157" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A157" s="1">
+        <v>46428.70833333333</v>
+      </c>
+    </row>
+    <row r="158" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A158" s="1">
+        <v>46429.70833333333</v>
+      </c>
+    </row>
+    <row r="159" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A159" s="1">
+        <v>46430.70833333333</v>
+      </c>
+    </row>
+    <row r="160" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A160" s="1">
+        <v>46431.70833333333</v>
+      </c>
+    </row>
+    <row r="161" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A161" s="1">
+        <v>46432.70833333333</v>
+      </c>
+    </row>
+    <row r="162" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A162" s="1">
+        <v>46433.70833333333</v>
+      </c>
+    </row>
+    <row r="163" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A163" s="1">
+        <v>46434.70833333333</v>
+      </c>
+    </row>
+    <row r="164" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A164" s="1">
+        <v>46435.70833333333</v>
+      </c>
+    </row>
+    <row r="165" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A165" s="1">
+        <v>46436.70833333333</v>
+      </c>
+    </row>
+    <row r="166" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A166" s="1">
+        <v>46437.70833333333</v>
+      </c>
+    </row>
+    <row r="167" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A167" s="1">
+        <v>46438.70833333333</v>
+      </c>
+    </row>
+    <row r="168" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A168" s="1">
+        <v>46439.70833333333</v>
+      </c>
+    </row>
+    <row r="169" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A169" s="1">
+        <v>46440.70833333333</v>
+      </c>
+    </row>
+    <row r="170" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A170" s="1">
+        <v>46441.70833333333</v>
+      </c>
+    </row>
+    <row r="171" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A171" s="1">
+        <v>46442.70833333333</v>
+      </c>
+    </row>
+    <row r="172" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A172" s="1">
+        <v>46443.70833333333</v>
+      </c>
+    </row>
+    <row r="173" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A173" s="1">
+        <v>46444.70833333333</v>
+      </c>
+    </row>
+    <row r="174" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A174" s="1">
+        <v>46445.70833333333</v>
+      </c>
+    </row>
+    <row r="175" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A175" s="1">
+        <v>46446.70833333333</v>
+      </c>
+    </row>
+    <row r="176" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A176" s="1">
+        <v>46447.70833333333</v>
+      </c>
+    </row>
+    <row r="177" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A177" s="1">
+        <v>46448.70833333333</v>
+      </c>
+    </row>
+    <row r="178" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A178" s="1">
+        <v>46449.70833333333</v>
+      </c>
+    </row>
+    <row r="179" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A179" s="1">
+        <v>46450.70833333333</v>
+      </c>
+    </row>
+    <row r="180" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A180" s="1">
+        <v>46451.70833333333</v>
+      </c>
+    </row>
+    <row r="181" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A181" s="1">
+        <v>46452.70833333333</v>
+      </c>
+    </row>
+    <row r="182" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A182" s="1">
+        <v>46453.70833333333</v>
+      </c>
+    </row>
+    <row r="183" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A183" s="1">
+        <v>46454.70833333333</v>
+      </c>
+    </row>
+    <row r="184" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A184" s="1">
+        <v>46455.70833333333</v>
+      </c>
+    </row>
+    <row r="185" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A185" s="1">
+        <v>46456.70833333333</v>
+      </c>
+    </row>
+    <row r="186" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A186" s="1">
+        <v>46457.70833333333</v>
+      </c>
+    </row>
+    <row r="187" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A187" s="1">
+        <v>46458.70833333333</v>
+      </c>
+    </row>
+    <row r="188" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A188" s="1">
+        <v>46459.70833333333</v>
+      </c>
+    </row>
+    <row r="189" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A189" s="1">
+        <v>46460.70833333333</v>
+      </c>
+    </row>
+    <row r="190" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A190" s="1">
+        <v>46461.70833333333</v>
+      </c>
+    </row>
+    <row r="191" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A191" s="1">
+        <v>46462.70833333333</v>
+      </c>
+    </row>
+    <row r="192" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A192" s="1">
+        <v>46463.70833333333</v>
+      </c>
+    </row>
+    <row r="193" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A193" s="1">
+        <v>46464.70833333333</v>
+      </c>
+    </row>
+    <row r="194" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A194" s="1">
+        <v>46465.70833333333</v>
+      </c>
+    </row>
+    <row r="195" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A195" s="1">
+        <v>46466.70833333333</v>
+      </c>
+    </row>
+    <row r="196" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A196" s="1">
+        <v>46467.70833333333</v>
+      </c>
+    </row>
+    <row r="197" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A197" s="1">
+        <v>46468.70833333333</v>
+      </c>
+    </row>
+    <row r="198" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A198" s="1">
+        <v>46469.70833333333</v>
+      </c>
+    </row>
+    <row r="199" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A199" s="1">
+        <v>46470.70833333333</v>
+      </c>
+    </row>
+    <row r="200" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A200" s="1">
+        <v>46471.70833333333</v>
+      </c>
+    </row>
+    <row r="201" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A201" s="1">
+        <v>46472.70833333333</v>
+      </c>
+    </row>
+    <row r="202" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A202" s="1">
+        <v>46473.70833333333</v>
+      </c>
+    </row>
+    <row r="203" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A203" s="1">
+        <v>46474.70833333333</v>
+      </c>
+    </row>
+    <row r="204" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A204" s="1">
+        <v>46475.70833333333</v>
+      </c>
+    </row>
+    <row r="205" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A205" s="1">
+        <v>46476.70833333333</v>
+      </c>
+    </row>
+    <row r="206" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A206" s="1">
+        <v>46477.70833333333</v>
+      </c>
+    </row>
+    <row r="207" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A207" s="1">
+        <v>46478.70833333333</v>
+      </c>
+    </row>
+    <row r="208" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A208" s="1">
+        <v>46479.70833333333</v>
+      </c>
+    </row>
+    <row r="209" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A209" s="1">
+        <v>46480.70833333333</v>
+      </c>
+    </row>
+    <row r="210" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A210" s="1">
+        <v>46481.70833333333</v>
+      </c>
+    </row>
+    <row r="211" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A211" s="1">
+        <v>46482.70833333333</v>
+      </c>
+    </row>
+    <row r="212" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A212" s="1">
+        <v>46483.70833333333</v>
+      </c>
+    </row>
+    <row r="213" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A213" s="1">
+        <v>46484.70833333333</v>
+      </c>
+    </row>
+    <row r="214" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A214" s="1">
+        <v>46485.70833333333</v>
+      </c>
+    </row>
+    <row r="215" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A215" s="1">
+        <v>46486.70833333333</v>
+      </c>
+    </row>
+    <row r="216" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A216" s="1">
+        <v>46487.70833333333</v>
+      </c>
+    </row>
+    <row r="217" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A217" s="1">
+        <v>46488.70833333333</v>
+      </c>
+    </row>
+    <row r="218" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A218" s="1">
+        <v>46489.70833333333</v>
+      </c>
+    </row>
+    <row r="219" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A219" s="1">
+        <v>46490.70833333333</v>
+      </c>
+    </row>
+    <row r="220" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A220" s="1">
+        <v>46491.70833333333</v>
+      </c>
+    </row>
+    <row r="221" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A221" s="1">
+        <v>46492.70833333333</v>
+      </c>
+    </row>
+    <row r="222" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A222" s="1">
+        <v>46493.70833333333</v>
+      </c>
+    </row>
+    <row r="223" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A223" s="1">
+        <v>46494.70833333333</v>
+      </c>
+    </row>
+    <row r="224" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A224" s="1">
+        <v>46495.70833333333</v>
+      </c>
+    </row>
+    <row r="225" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A225" s="1">
+        <v>46496.70833333333</v>
+      </c>
+    </row>
+    <row r="226" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A226" s="1">
+        <v>46497.70833333333</v>
+      </c>
+    </row>
+    <row r="227" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A227" s="1">
+        <v>46498.70833333333</v>
+      </c>
+    </row>
+    <row r="228" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A228" s="1">
+        <v>46499.70833333333</v>
+      </c>
+    </row>
+    <row r="229" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A229" s="1">
+        <v>46500.70833333333</v>
+      </c>
+    </row>
+    <row r="230" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A230" s="1">
+        <v>46501.70833333333</v>
+      </c>
+    </row>
+    <row r="231" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A231" s="1">
+        <v>46502.70833333333</v>
+      </c>
+    </row>
+    <row r="232" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A232" s="1">
+        <v>46503.70833333333</v>
+      </c>
+    </row>
+    <row r="233" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A233" s="1">
+        <v>46504.70833333333</v>
+      </c>
+    </row>
+    <row r="234" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A234" s="1">
+        <v>46505.70833333333</v>
+      </c>
+    </row>
+    <row r="235" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A235" s="1">
+        <v>46506.70833333333</v>
+      </c>
+    </row>
+    <row r="236" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A236" s="1">
+        <v>46507.70833333333</v>
+      </c>
+    </row>
+    <row r="237" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A237" s="1">
+        <v>46508.70833333333</v>
+      </c>
+    </row>
+    <row r="238" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A238" s="1">
+        <v>46509.70833333333</v>
+      </c>
+    </row>
+    <row r="239" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A239" s="1">
+        <v>46510.70833333333</v>
+      </c>
+    </row>
+    <row r="240" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A240" s="1">
+        <v>46511.70833333333</v>
+      </c>
+    </row>
+    <row r="241" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A241" s="1">
+        <v>46512.70833333333</v>
+      </c>
+    </row>
+    <row r="242" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A242" s="1">
+        <v>46513.70833333333</v>
+      </c>
+    </row>
+    <row r="243" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A243" s="1">
+        <v>46514.70833333333</v>
+      </c>
+    </row>
+    <row r="244" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A244" s="1">
+        <v>46515.70833333333</v>
+      </c>
+    </row>
+    <row r="245" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A245" s="1">
+        <v>46516.70833333333</v>
+      </c>
+    </row>
+    <row r="246" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A246" s="1">
+        <v>46517.70833333333</v>
+      </c>
+    </row>
+    <row r="247" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A247" s="1">
+        <v>46518.70833333333</v>
+      </c>
+    </row>
+    <row r="248" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A248" s="1">
+        <v>46519.70833333333</v>
+      </c>
+    </row>
+    <row r="249" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A249" s="1">
+        <v>46520.70833333333</v>
+      </c>
+    </row>
+    <row r="250" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A250" s="1">
+        <v>46521.70833333333</v>
+      </c>
+    </row>
+    <row r="251" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A251" s="1">
+        <v>46522.70833333333</v>
+      </c>
+    </row>
+    <row r="252" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A252" s="1">
+        <v>46523.70833333333</v>
+      </c>
+    </row>
+    <row r="253" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A253" s="1">
+        <v>46524.70833333333</v>
+      </c>
+    </row>
+    <row r="254" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A254" s="1">
+        <v>46525.70833333333</v>
+      </c>
+    </row>
+    <row r="255" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A255" s="1">
+        <v>46526.70833333333</v>
+      </c>
+    </row>
+    <row r="256" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A256" s="1">
+        <v>46527.70833333333</v>
+      </c>
+    </row>
+    <row r="257" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A257" s="1">
+        <v>46528.70833333333</v>
+      </c>
+    </row>
+    <row r="258" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A258" s="1">
+        <v>46529.70833333333</v>
+      </c>
+    </row>
+    <row r="259" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A259" s="1">
+        <v>46530.70833333333</v>
+      </c>
+    </row>
+    <row r="260" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A260" s="1">
+        <v>46531.70833333333</v>
+      </c>
+    </row>
+    <row r="261" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A261" s="1">
+        <v>46532.70833333333</v>
+      </c>
+    </row>
+    <row r="262" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A262" s="1">
+        <v>46533.70833333333</v>
+      </c>
+    </row>
+    <row r="263" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A263" s="1">
+        <v>46534.70833333333</v>
+      </c>
+    </row>
+    <row r="264" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A264" s="1">
+        <v>46535.70833333333</v>
+      </c>
+    </row>
+    <row r="265" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A265" s="1">
+        <v>46536.70833333333</v>
+      </c>
+    </row>
+    <row r="266" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A266" s="1">
+        <v>46537.70833333333</v>
+      </c>
+    </row>
+    <row r="267" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A267" s="1">
+        <v>46538.70833333333</v>
+      </c>
+    </row>
+    <row r="268" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A268" s="1">
+        <v>46539.70833333333</v>
+      </c>
+    </row>
+    <row r="269" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A269" s="1">
+        <v>46540.70833333333</v>
+      </c>
+    </row>
+    <row r="270" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A270" s="1">
+        <v>46541.70833333333</v>
+      </c>
+    </row>
+    <row r="271" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A271" s="1">
+        <v>46542.70833333333</v>
+      </c>
+    </row>
+    <row r="272" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A272" s="1">
+        <v>46543.70833333333</v>
+      </c>
+    </row>
+    <row r="273" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A273" s="1">
+        <v>46544.70833333333</v>
+      </c>
+    </row>
+    <row r="274" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A274" s="1">
+        <v>46545.70833333333</v>
+      </c>
+    </row>
+    <row r="275" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A275" s="1">
+        <v>46546.70833333333</v>
+      </c>
+    </row>
+    <row r="276" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A276" s="1">
+        <v>46547.70833333333</v>
+      </c>
+    </row>
+    <row r="277" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A277" s="1">
+        <v>46548.70833333333</v>
+      </c>
+    </row>
+    <row r="278" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A278" s="1">
+        <v>46549.70833333333</v>
+      </c>
+    </row>
+    <row r="279" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A279" s="1">
+        <v>46550.70833333333</v>
+      </c>
+    </row>
+    <row r="280" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A280" s="1">
+        <v>46551.70833333333</v>
+      </c>
+    </row>
+    <row r="281" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A281" s="1">
+        <v>46552.70833333333</v>
+      </c>
+    </row>
+    <row r="282" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A282" s="1">
+        <v>46553.70833333333</v>
+      </c>
+    </row>
+    <row r="283" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A283" s="1">
+        <v>46554.70833333333</v>
+      </c>
+    </row>
+    <row r="284" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A284" s="1">
+        <v>46555.70833333333</v>
+      </c>
+    </row>
+    <row r="285" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A285" s="1">
+        <v>46556.70833333333</v>
+      </c>
+    </row>
+    <row r="286" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A286" s="1">
+        <v>46557.70833333333</v>
+      </c>
+    </row>
+    <row r="287" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A287" s="1">
+        <v>46558.70833333333</v>
+      </c>
+    </row>
+    <row r="288" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A288" s="1">
+        <v>46559.70833333333</v>
+      </c>
+    </row>
+    <row r="289" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A289" s="1">
+        <v>46560.70833333333</v>
+      </c>
+    </row>
+    <row r="290" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A290" s="1">
+        <v>46561.70833333333</v>
+      </c>
+    </row>
+    <row r="291" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A291" s="1">
+        <v>46562.70833333333</v>
+      </c>
+    </row>
+    <row r="292" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A292" s="1">
+        <v>46563.70833333333</v>
+      </c>
+    </row>
+    <row r="293" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A293" s="1">
+        <v>46564.70833333333</v>
+      </c>
+    </row>
+    <row r="294" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A294" s="1">
+        <v>46565.70833333333</v>
+      </c>
+    </row>
+    <row r="295" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A295" s="1">
+        <v>46566.70833333333</v>
+      </c>
+    </row>
+    <row r="296" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A296" s="1">
+        <v>46567.70833333333</v>
+      </c>
+    </row>
+    <row r="297" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A297" s="1">
+        <v>46568.70833333333</v>
+      </c>
+    </row>
+    <row r="298" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A298" s="1">
+        <v>46569.70833333333</v>
+      </c>
+    </row>
+    <row r="299" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A299" s="1">
+        <v>46570.70833333333</v>
+      </c>
+    </row>
+    <row r="300" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A300" s="1">
+        <v>46571.70833333333</v>
       </c>
     </row>
   </sheetData>
@@ -852,7 +2381,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:B18"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
@@ -861,147 +2390,147 @@
     <col min="2" max="2" width="80" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" s="8" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="8" t="s">
+    <row r="1" spans="1:2" s="12" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="12" t="s">
         <v>37</v>
       </c>
-      <c r="B1" s="8" t="s">
+      <c r="B1" s="12" t="s">
         <v>38</v>
       </c>
     </row>
-    <row r="2" spans="1:2" s="9" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="9" t="s">
-        <v>22</v>
-      </c>
-      <c r="B2" s="9" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="3" spans="1:2" s="9" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="9" t="s">
+    <row r="2" spans="1:2" s="13" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A2" s="13" t="s">
+        <v>22</v>
+      </c>
+      <c r="B2" s="13" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" s="13" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A3" s="13" t="s">
         <v>39</v>
       </c>
-      <c r="B3" s="9" t="s">
+      <c r="B3" s="13" t="s">
         <v>40</v>
       </c>
     </row>
-    <row r="4" spans="1:2" s="9" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="9" t="s">
+    <row r="4" spans="1:2" s="13" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A4" s="13" t="s">
         <v>41</v>
       </c>
-      <c r="B4" s="9" t="s">
+      <c r="B4" s="13" t="s">
         <v>42</v>
       </c>
     </row>
-    <row r="5" spans="1:2" s="9" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="9" t="s">
+    <row r="5" spans="1:2" s="13" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A5" s="13" t="s">
         <v>43</v>
       </c>
-      <c r="B5" s="9" t="s">
+      <c r="B5" s="13" t="s">
         <v>44</v>
       </c>
     </row>
-    <row r="6" spans="1:2" s="9" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="9" t="s">
+    <row r="6" spans="1:2" s="13" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A6" s="13" t="s">
         <v>45</v>
       </c>
-      <c r="B6" s="9" t="s">
+      <c r="B6" s="13" t="s">
         <v>46</v>
       </c>
     </row>
-    <row r="7" spans="1:2" s="9" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="9" t="s">
-        <v>22</v>
-      </c>
-      <c r="B7" s="9" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="8" spans="1:2" s="8" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="8" t="s">
+    <row r="7" spans="1:2" s="13" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A7" s="13" t="s">
+        <v>22</v>
+      </c>
+      <c r="B7" s="13" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2" s="12" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A8" s="12" t="s">
         <v>47</v>
       </c>
-      <c r="B8" s="8" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="9" spans="1:2" s="9" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="9" t="s">
+      <c r="B8" s="12" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2" s="13" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A9" s="13" t="s">
         <v>11</v>
       </c>
-      <c r="B9" s="9" t="s">
+      <c r="B9" s="13" t="s">
         <v>48</v>
       </c>
     </row>
-    <row r="10" spans="1:2" s="9" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="9" t="s">
+    <row r="10" spans="1:2" s="13" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A10" s="13" t="s">
         <v>12</v>
       </c>
-      <c r="B10" s="9" t="s">
+      <c r="B10" s="13" t="s">
         <v>48</v>
       </c>
     </row>
-    <row r="11" spans="1:2" s="9" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="9" t="s">
+    <row r="11" spans="1:2" s="13" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A11" s="13" t="s">
         <v>13</v>
       </c>
-      <c r="B11" s="9" t="s">
+      <c r="B11" s="13" t="s">
         <v>49</v>
       </c>
     </row>
-    <row r="12" spans="1:2" s="9" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="9" t="s">
+    <row r="12" spans="1:2" s="13" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A12" s="13" t="s">
         <v>14</v>
       </c>
-      <c r="B12" s="9" t="s">
+      <c r="B12" s="13" t="s">
         <v>49</v>
       </c>
     </row>
-    <row r="13" spans="1:2" s="9" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="9" t="s">
+    <row r="13" spans="1:2" s="13" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A13" s="13" t="s">
         <v>15</v>
       </c>
-      <c r="B13" s="9" t="s">
+      <c r="B13" s="13" t="s">
         <v>49</v>
       </c>
     </row>
-    <row r="14" spans="1:2" s="9" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="9" t="s">
+    <row r="14" spans="1:2" s="13" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A14" s="13" t="s">
         <v>16</v>
       </c>
-      <c r="B14" s="9" t="s">
+      <c r="B14" s="13" t="s">
         <v>50</v>
       </c>
     </row>
-    <row r="15" spans="1:2" s="9" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="9" t="s">
+    <row r="15" spans="1:2" s="13" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A15" s="13" t="s">
         <v>17</v>
       </c>
-      <c r="B15" s="9" t="s">
+      <c r="B15" s="13" t="s">
         <v>48</v>
       </c>
     </row>
-    <row r="16" spans="1:2" s="9" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="9" t="s">
+    <row r="16" spans="1:2" s="13" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A16" s="13" t="s">
         <v>51</v>
       </c>
-      <c r="B16" s="9" t="s">
+      <c r="B16" s="13" t="s">
         <v>52</v>
       </c>
     </row>
-    <row r="17" spans="1:2" s="9" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A17" s="9" t="s">
+    <row r="17" spans="1:2" s="13" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A17" s="13" t="s">
         <v>53</v>
       </c>
-      <c r="B17" s="9" t="s">
+      <c r="B17" s="13" t="s">
         <v>52</v>
       </c>
     </row>
-    <row r="18" spans="1:2" s="9" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A18" s="9" t="s">
+    <row r="18" spans="1:2" s="13" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A18" s="13" t="s">
         <v>54</v>
       </c>
-      <c r="B18" s="9" t="s">
+      <c r="B18" s="13" t="s">
         <v>48</v>
       </c>
     </row>

</xml_diff>